<commit_message>
chore: fixed 128 minor n elec list
</commit_message>
<xml_diff>
--- a/raw/time_tables/B.Tech 128 (btech-128)/5/1.xlsx
+++ b/raw/time_tables/B.Tech 128 (btech-128)/5/1.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="500" uniqueCount="406">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="548" uniqueCount="434">
   <si>
     <t>B. Tech.  III Yr(V SEMESTER) TIMETABLE ODD SEMESTER 2026, JIIT-128</t>
   </si>
@@ -486,22 +486,121 @@
     <t>LF11F12(24B11CS312)-CR54/SAP</t>
   </si>
   <si>
-    <t>FRIDAY</t>
+    <t>THURSDAY</t>
   </si>
   <si>
     <t>LALL(17B1NMA533)-3083/SREYA</t>
   </si>
   <si>
-    <t>LF5F6(20B13HS311) -226/PRV</t>
+    <t>PF13F14(24B15CS313) -CL4/ARM/NISHANT</t>
   </si>
   <si>
     <t>LALL(19B12CS426)-111
 /NFCS22</t>
   </si>
   <si>
+    <t>LALL(17B1NEC735)-226 /RUS</t>
+  </si>
+  <si>
     <t>LALL(16B1NMA533)-259/AMB</t>
   </si>
   <si>
+    <t>P F13(24B15CS314)-CR104/NFCS21</t>
+  </si>
+  <si>
+    <t>P F10F11F12(24B15CS312) -CL3/ANU/TWT/NRP/AKS/ARM</t>
+  </si>
+  <si>
+    <t>LALL(26B42EC313) -230/HIG</t>
+  </si>
+  <si>
+    <t>P F14(24B15CS314)-3121/NFCS22</t>
+  </si>
+  <si>
+    <t>PE4(24B45EC311)-142/RAP</t>
+  </si>
+  <si>
+    <t>LALL(17B1NMA531)-CR54/PKS</t>
+  </si>
+  <si>
+    <t>LF7F8(24B11CS312) -244/AMS</t>
+  </si>
+  <si>
+    <t>PF16F17(24B25CS315) -CR99/AKH/NFCS2/NFCS23/NFCS26</t>
+  </si>
+  <si>
+    <t>PE3(18B15EC212)-256A/PAA</t>
+  </si>
+  <si>
+    <t>LALL (16B1NPH531) -3093 /KAS</t>
+  </si>
+  <si>
+    <t>LF11F12(24B11CS312) - 259/SAP</t>
+  </si>
+  <si>
+    <t>PF7F8F9(24B15CS313) -CL3/MGO/DRHUV/HMA/PKM</t>
+  </si>
+  <si>
+    <t>LF7F8(24B11CS313) -CR54/PKM</t>
+  </si>
+  <si>
+    <t>LF18F19(24B11CS313) -138/AKH</t>
+  </si>
+  <si>
+    <t>PF1F2F3F4F5F6F18F19(26B16CS313)-CL4/AKB/PSK</t>
+  </si>
+  <si>
+    <t>PF1F2F3F13F14F16F17F18F19(26B16CS317)-CR104/SAP/PKM/NF30</t>
+  </si>
+  <si>
+    <t>LALL (16B1NPH535) -3098 /ANK</t>
+  </si>
+  <si>
+    <t>LF13F14(24B11CS313) -153/DVG</t>
+  </si>
+  <si>
+    <t>LF11F12(24B11CS313) -230 /MADHAV</t>
+  </si>
+  <si>
+    <t>LE3E4(24B41EC311)- 226/ANG</t>
+  </si>
+  <si>
+    <t>LF5F6(20B13HS311) -259/PRV</t>
+  </si>
+  <si>
+    <t>LALL (26B12PH312) - 230/SKA</t>
+  </si>
+  <si>
+    <t>TE2(24B41EC311)- 225/ANG</t>
+  </si>
+  <si>
+    <t>TF10(24B11CS313)-138/NISHANT</t>
+  </si>
+  <si>
+    <t>LE1E2(18B11EC212) -230/PAA</t>
+  </si>
+  <si>
+    <t>LF3F4(20B13HS311) -230/SAK</t>
+  </si>
+  <si>
+    <t>TE1(18B11EC212) -229/PAA</t>
+  </si>
+  <si>
+    <t>LF5F6(24B11CS313) -226/HMA</t>
+  </si>
+  <si>
+    <t>LF9F10(24B11CS312)-3083/TWT</t>
+  </si>
+  <si>
+    <t>TF9(24B11CS313)-CR54/VAISHNAVI</t>
+  </si>
+  <si>
+    <t>FRIDAY</t>
+  </si>
+  <si>
+    <t>LF5F6(20B13HS311) -226/PRV</t>
+  </si>
+  <si>
     <t>P F18 F19(24B15CS313) -CR99/HMA/MINAL/NISHANT</t>
   </si>
   <si>
@@ -517,9 +616,6 @@
     <t>PF1F2F11F12F16F17F18F19(26B16CS318)-CR99/-BHB/JSH/NFCS31</t>
   </si>
   <si>
-    <t>LALL(17B1NMA531)-CR54/PKS</t>
-  </si>
-  <si>
     <t>PF7F8F9F10F11F12F13F14F16F17(24B16CS313)-CL4/-AKB/PSK</t>
   </si>
   <si>
@@ -529,9 +625,6 @@
     <t>PF1F2F3F13F14F16F17F18(26B16CS316)-CR104/-RKB/NFCS36</t>
   </si>
   <si>
-    <t>LALL (16B1NPH531) -3093 /KAS</t>
-  </si>
-  <si>
     <t>LE3E4(24B41EC311)- 230/ANG</t>
   </si>
   <si>
@@ -553,9 +646,6 @@
     <t>PF7F8F18(24B16CS320)-3067/-PRY</t>
   </si>
   <si>
-    <t>LALL (16B1NPH535) -3098 /ANK</t>
-  </si>
-  <si>
     <t>TF5(24B11CS313)-CR54/PKM</t>
   </si>
   <si>
@@ -565,9 +655,6 @@
     <t>PF12F13F14F16F17F19(24B16CS320)-3121/NFCS37</t>
   </si>
   <si>
-    <t>LALL (26B12PH312) - 230/SKA</t>
-  </si>
-  <si>
     <t>TF6(24B11CS313)-244VAISHNAVI</t>
   </si>
   <si>
@@ -599,9 +686,6 @@
   </si>
   <si>
     <t>LF16F17(20B13HS311) -226/SHV</t>
-  </si>
-  <si>
-    <t>LALL(26B42EC313) -230/HIG</t>
   </si>
   <si>
     <t>TF16(24B11CS313)-138/NISHANT</t>
@@ -2149,71 +2233,80 @@
         <v>150</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>96</v>
+        <v>143</v>
       </c>
       <c r="E43" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="H43" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="F43" s="1" t="s">
-        <v>117</v>
+      <c r="J43" s="1" t="s">
+        <v>73</v>
       </c>
       <c r="K43" s="1" t="s">
         <v>152</v>
       </c>
     </row>
     <row r="44" ht="15.75" customHeight="1">
+      <c r="B44" s="1" t="s">
+        <v>153</v>
+      </c>
       <c r="C44" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="F44" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="E44" s="1" t="s">
         <v>155</v>
       </c>
+      <c r="H44" s="1" t="s">
+        <v>156</v>
+      </c>
     </row>
     <row r="45" ht="15.75" customHeight="1">
+      <c r="B45" s="1" t="s">
+        <v>157</v>
+      </c>
       <c r="C45" s="1" t="s">
         <v>119</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>156</v>
-      </c>
-      <c r="F45" s="1" t="s">
-        <v>157</v>
+        <v>121</v>
+      </c>
+      <c r="E45" s="1" t="s">
+        <v>158</v>
       </c>
       <c r="H45" s="1" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="46" ht="15.75" customHeight="1">
       <c r="C46" s="1" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="F46" s="1" t="s">
         <v>161</v>
       </c>
+      <c r="E46" s="1" t="s">
+        <v>162</v>
+      </c>
       <c r="H46" s="1" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="47" ht="15.75" customHeight="1">
       <c r="C47" s="1" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="E47" s="1" t="s">
-        <v>165</v>
-      </c>
-      <c r="F47" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="H47" s="1" t="s">
+      <c r="I47" s="1" t="s">
         <v>167</v>
       </c>
     </row>
@@ -2224,7 +2317,7 @@
       <c r="D48" s="1" t="s">
         <v>168</v>
       </c>
-      <c r="F48" s="1" t="s">
+      <c r="E48" s="1" t="s">
         <v>169</v>
       </c>
       <c r="H48" s="1" t="s">
@@ -2238,1053 +2331,1199 @@
       <c r="D49" s="1" t="s">
         <v>172</v>
       </c>
+      <c r="E49" s="1" t="s">
+        <v>173</v>
+      </c>
       <c r="F49" s="1" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="H49" s="1" t="s">
-        <v>174</v>
+        <v>19</v>
+      </c>
+      <c r="I49" s="1" t="s">
+        <v>175</v>
       </c>
     </row>
     <row r="50" ht="15.75" customHeight="1">
       <c r="C50" s="1" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="D50" s="1" t="s">
-        <v>176</v>
+        <v>177</v>
+      </c>
+      <c r="E50" s="1" t="s">
+        <v>178</v>
       </c>
       <c r="F50" s="1" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="H50" s="1" t="s">
-        <v>54</v>
+        <v>71</v>
       </c>
       <c r="I50" s="1" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="51" ht="15.75" customHeight="1">
       <c r="C51" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="F51" s="1" t="s">
-        <v>179</v>
+      <c r="D51" s="1" t="s">
+        <v>181</v>
       </c>
       <c r="H51" s="1" t="s">
-        <v>180</v>
+        <v>90</v>
       </c>
       <c r="I51" s="1" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
     <row r="52" ht="15.75" customHeight="1">
       <c r="C52" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="F52" s="1" t="s">
-        <v>182</v>
+      <c r="D52" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="H52" s="1" t="s">
+        <v>184</v>
       </c>
     </row>
     <row r="53" ht="15.75" customHeight="1"/>
-    <row r="54" ht="15.75" customHeight="1"/>
+    <row r="54" ht="15.75" customHeight="1">
+      <c r="A54" s="1" t="s">
+        <v>185</v>
+      </c>
+    </row>
     <row r="55" ht="15.75" customHeight="1">
-      <c r="A55" s="1" t="s">
-        <v>183</v>
+      <c r="C55" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="D55" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="E55" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="F55" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="K55" s="1" t="s">
+        <v>152</v>
       </c>
     </row>
     <row r="56" ht="15.75" customHeight="1">
+      <c r="C56" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="D56" s="1" t="s">
+        <v>187</v>
+      </c>
       <c r="F56" s="1" t="s">
-        <v>184</v>
+        <v>188</v>
       </c>
     </row>
     <row r="57" ht="15.75" customHeight="1">
-      <c r="B57" s="1" t="s">
-        <v>185</v>
-      </c>
       <c r="C57" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="E57" s="1" t="s">
-        <v>186</v>
+        <v>119</v>
+      </c>
+      <c r="D57" s="1" t="s">
+        <v>189</v>
       </c>
       <c r="F57" s="1" t="s">
-        <v>151</v>
+        <v>190</v>
+      </c>
+      <c r="H57" s="1" t="s">
+        <v>191</v>
       </c>
     </row>
     <row r="58" ht="15.75" customHeight="1">
-      <c r="B58" s="1" t="s">
-        <v>187</v>
-      </c>
       <c r="C58" s="1" t="s">
-        <v>115</v>
+        <v>160</v>
       </c>
       <c r="D58" s="1" t="s">
-        <v>188</v>
-      </c>
-      <c r="E58" s="1" t="s">
-        <v>96</v>
+        <v>192</v>
       </c>
       <c r="F58" s="1" t="s">
-        <v>189</v>
+        <v>193</v>
+      </c>
+      <c r="H58" s="1" t="s">
+        <v>194</v>
       </c>
     </row>
     <row r="59" ht="15.75" customHeight="1">
-      <c r="B59" s="1" t="s">
-        <v>190</v>
+      <c r="C59" s="1" t="s">
+        <v>164</v>
       </c>
       <c r="D59" s="1" t="s">
-        <v>191</v>
+        <v>195</v>
+      </c>
+      <c r="E59" s="1" t="s">
+        <v>196</v>
       </c>
       <c r="F59" s="1" t="s">
-        <v>192</v>
+        <v>197</v>
+      </c>
+      <c r="H59" s="1" t="s">
+        <v>198</v>
       </c>
     </row>
     <row r="60" ht="15.75" customHeight="1">
-      <c r="B60" s="1" t="s">
-        <v>193</v>
+      <c r="C60" s="1" t="s">
+        <v>131</v>
       </c>
       <c r="D60" s="1" t="s">
-        <v>194</v>
+        <v>199</v>
       </c>
       <c r="F60" s="1" t="s">
-        <v>195</v>
+        <v>200</v>
+      </c>
+      <c r="H60" s="1" t="s">
+        <v>201</v>
       </c>
     </row>
     <row r="61" ht="15.75" customHeight="1">
-      <c r="B61" s="1" t="s">
-        <v>196</v>
+      <c r="C61" s="1" t="s">
+        <v>171</v>
       </c>
       <c r="D61" s="1" t="s">
-        <v>197</v>
+        <v>202</v>
       </c>
       <c r="F61" s="1" t="s">
-        <v>198</v>
+        <v>203</v>
+      </c>
+      <c r="H61" s="1" t="s">
+        <v>204</v>
       </c>
     </row>
     <row r="62" ht="15.75" customHeight="1">
-      <c r="B62" s="1" t="s">
-        <v>199</v>
+      <c r="C62" s="1" t="s">
+        <v>176</v>
       </c>
       <c r="D62" s="1" t="s">
-        <v>200</v>
+        <v>205</v>
       </c>
       <c r="F62" s="1" t="s">
-        <v>201</v>
+        <v>206</v>
+      </c>
+      <c r="H62" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="I62" s="1" t="s">
+        <v>207</v>
       </c>
     </row>
     <row r="63" ht="15.75" customHeight="1">
-      <c r="D63" s="1" t="s">
-        <v>202</v>
+      <c r="C63" s="1" t="s">
+        <v>144</v>
       </c>
       <c r="F63" s="1" t="s">
-        <v>203</v>
+        <v>208</v>
+      </c>
+      <c r="H63" s="1" t="s">
+        <v>209</v>
+      </c>
+      <c r="I63" s="1" t="s">
+        <v>210</v>
       </c>
     </row>
     <row r="64" ht="15.75" customHeight="1">
-      <c r="D64" s="1" t="s">
-        <v>204</v>
+      <c r="C64" s="1" t="s">
+        <v>147</v>
       </c>
       <c r="F64" s="1" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="65" ht="15.75" customHeight="1">
-      <c r="D65" s="1" t="s">
-        <v>205</v>
-      </c>
-      <c r="E65" s="1" t="s">
-        <v>206</v>
-      </c>
-      <c r="F65" s="1" t="s">
-        <v>53</v>
-      </c>
-    </row>
+        <v>211</v>
+      </c>
+    </row>
+    <row r="65" ht="15.75" customHeight="1"/>
     <row r="66" ht="15.75" customHeight="1"/>
     <row r="67" ht="15.75" customHeight="1">
-      <c r="B67" s="1" t="s">
-        <v>207</v>
-      </c>
-      <c r="C67" s="1" t="s">
-        <v>208</v>
-      </c>
-      <c r="D67" s="1" t="s">
-        <v>207</v>
-      </c>
-      <c r="E67" s="1" t="s">
-        <v>208</v>
-      </c>
-      <c r="F67" s="1" t="s">
-        <v>207</v>
-      </c>
-      <c r="G67" s="1" t="s">
-        <v>208</v>
-      </c>
-      <c r="H67" s="1" t="s">
-        <v>209</v>
-      </c>
-      <c r="I67" s="1" t="s">
-        <v>210</v>
-      </c>
-      <c r="J67" s="1" t="s">
-        <v>209</v>
-      </c>
-      <c r="K67" s="1" t="s">
-        <v>210</v>
+      <c r="A67" s="1" t="s">
+        <v>212</v>
       </c>
     </row>
     <row r="68" ht="15.75" customHeight="1">
-      <c r="B68" s="1" t="s">
-        <v>211</v>
-      </c>
-      <c r="C68" s="1" t="s">
-        <v>212</v>
-      </c>
-      <c r="E68" s="1" t="s">
+      <c r="F68" s="1" t="s">
         <v>213</v>
-      </c>
-      <c r="F68" s="1" t="s">
-        <v>214</v>
-      </c>
-      <c r="G68" s="1" t="s">
-        <v>215</v>
-      </c>
-      <c r="H68" s="1" t="s">
-        <v>216</v>
-      </c>
-      <c r="I68" s="1" t="s">
-        <v>217</v>
-      </c>
-      <c r="J68" s="1" t="s">
-        <v>218</v>
-      </c>
-      <c r="K68" s="1" t="s">
-        <v>219</v>
       </c>
     </row>
     <row r="69" ht="15.75" customHeight="1">
       <c r="B69" s="1" t="s">
-        <v>220</v>
+        <v>214</v>
       </c>
       <c r="C69" s="1" t="s">
-        <v>221</v>
-      </c>
-      <c r="D69" s="1" t="s">
-        <v>222</v>
+        <v>111</v>
       </c>
       <c r="E69" s="1" t="s">
-        <v>223</v>
+        <v>215</v>
       </c>
       <c r="F69" s="1" t="s">
-        <v>224</v>
-      </c>
-      <c r="G69" s="1" t="s">
-        <v>225</v>
-      </c>
-      <c r="H69" s="1" t="s">
-        <v>226</v>
-      </c>
-      <c r="I69" s="1" t="s">
-        <v>227</v>
-      </c>
-      <c r="J69" s="1" t="s">
-        <v>228</v>
-      </c>
-      <c r="K69" s="1" t="s">
-        <v>229</v>
+        <v>186</v>
       </c>
     </row>
     <row r="70" ht="15.75" customHeight="1">
       <c r="B70" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="C70" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="D70" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="E70" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="F70" s="1" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="71" ht="15.75" customHeight="1">
+      <c r="B71" s="1" t="s">
+        <v>218</v>
+      </c>
+      <c r="D71" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="F71" s="1" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="72" ht="15.75" customHeight="1">
+      <c r="B72" s="1" t="s">
+        <v>221</v>
+      </c>
+      <c r="D72" s="1" t="s">
+        <v>222</v>
+      </c>
+      <c r="F72" s="1" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="73" ht="15.75" customHeight="1">
+      <c r="B73" s="1" t="s">
+        <v>224</v>
+      </c>
+      <c r="D73" s="1" t="s">
+        <v>225</v>
+      </c>
+      <c r="F73" s="1" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="74" ht="15.75" customHeight="1">
+      <c r="B74" s="1" t="s">
+        <v>227</v>
+      </c>
+      <c r="D74" s="1" t="s">
+        <v>228</v>
+      </c>
+      <c r="F74" s="1" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="75" ht="15.75" customHeight="1">
+      <c r="D75" s="1" t="s">
         <v>230</v>
       </c>
-      <c r="C70" s="1" t="s">
+      <c r="F75" s="1" t="s">
         <v>231</v>
       </c>
-      <c r="D70" s="1" t="s">
+    </row>
+    <row r="76" ht="15.75" customHeight="1">
+      <c r="D76" s="1" t="s">
         <v>232</v>
       </c>
-      <c r="E70" s="1" t="s">
+      <c r="F76" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="77" ht="15.75" customHeight="1">
+      <c r="D77" s="1" t="s">
         <v>233</v>
       </c>
-      <c r="F70" s="1" t="s">
+      <c r="E77" s="1" t="s">
         <v>234</v>
       </c>
-      <c r="G70" s="1" t="s">
+      <c r="F77" s="1" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="78" ht="15.75" customHeight="1"/>
+    <row r="79" ht="15.75" customHeight="1">
+      <c r="B79" s="1" t="s">
         <v>235</v>
       </c>
-      <c r="H70" s="1" t="s">
+      <c r="C79" s="1" t="s">
         <v>236</v>
       </c>
-      <c r="I70" s="1" t="s">
+      <c r="D79" s="1" t="s">
+        <v>235</v>
+      </c>
+      <c r="E79" s="1" t="s">
+        <v>236</v>
+      </c>
+      <c r="F79" s="1" t="s">
+        <v>235</v>
+      </c>
+      <c r="G79" s="1" t="s">
+        <v>236</v>
+      </c>
+      <c r="H79" s="1" t="s">
         <v>237</v>
       </c>
-      <c r="J70" s="1" t="s">
+      <c r="I79" s="1" t="s">
         <v>238</v>
       </c>
-      <c r="K70" s="1" t="s">
-        <v>239</v>
-      </c>
-    </row>
-    <row r="71" ht="15.75" customHeight="1">
-      <c r="C71" s="1" t="s">
-        <v>240</v>
-      </c>
-      <c r="E71" s="1" t="s">
-        <v>241</v>
-      </c>
-      <c r="F71" s="1" t="s">
-        <v>242</v>
-      </c>
-      <c r="G71" s="1" t="s">
-        <v>243</v>
-      </c>
-      <c r="H71" s="1" t="s">
-        <v>244</v>
-      </c>
-      <c r="I71" s="1" t="s">
-        <v>245</v>
-      </c>
-      <c r="J71" s="1" t="s">
-        <v>246</v>
-      </c>
-      <c r="K71" s="1" t="s">
-        <v>247</v>
-      </c>
-    </row>
-    <row r="72" ht="15.75" customHeight="1">
-      <c r="C72" s="1" t="s">
-        <v>248</v>
-      </c>
-      <c r="E72" s="1" t="s">
-        <v>249</v>
-      </c>
-      <c r="F72" s="1" t="s">
-        <v>250</v>
-      </c>
-      <c r="G72" s="1" t="s">
-        <v>251</v>
-      </c>
-      <c r="H72" s="1" t="s">
-        <v>252</v>
-      </c>
-      <c r="I72" s="1" t="s">
-        <v>253</v>
-      </c>
-      <c r="J72" s="1" t="s">
-        <v>254</v>
-      </c>
-      <c r="K72" s="1" t="s">
-        <v>255</v>
-      </c>
-    </row>
-    <row r="73" ht="15.75" customHeight="1">
-      <c r="C73" s="1" t="s">
-        <v>240</v>
-      </c>
-      <c r="E73" s="1" t="s">
-        <v>256</v>
-      </c>
-      <c r="F73" s="1" t="s">
-        <v>257</v>
-      </c>
-      <c r="G73" s="1" t="s">
-        <v>258</v>
-      </c>
-      <c r="H73" s="1" t="s">
-        <v>259</v>
-      </c>
-      <c r="I73" s="1" t="s">
-        <v>260</v>
-      </c>
-      <c r="J73" s="1" t="s">
-        <v>261</v>
-      </c>
-      <c r="K73" s="1" t="s">
-        <v>262</v>
-      </c>
-    </row>
-    <row r="74" ht="15.75" customHeight="1">
-      <c r="C74" s="1" t="s">
-        <v>248</v>
-      </c>
-      <c r="E74" s="1" t="s">
-        <v>263</v>
-      </c>
-      <c r="F74" s="1" t="s">
-        <v>264</v>
-      </c>
-      <c r="G74" s="1" t="s">
-        <v>265</v>
-      </c>
-      <c r="H74" s="1" t="s">
-        <v>259</v>
-      </c>
-      <c r="I74" s="1" t="s">
-        <v>260</v>
-      </c>
-      <c r="J74" s="1" t="s">
-        <v>266</v>
-      </c>
-      <c r="K74" s="1" t="s">
-        <v>267</v>
-      </c>
-    </row>
-    <row r="75" ht="15.75" customHeight="1">
-      <c r="B75" s="1" t="s">
-        <v>268</v>
-      </c>
-      <c r="C75" s="1" t="s">
-        <v>269</v>
-      </c>
-      <c r="D75" s="1" t="s">
-        <v>270</v>
-      </c>
-      <c r="E75" s="1" t="s">
-        <v>271</v>
-      </c>
-      <c r="F75" s="1" t="s">
-        <v>272</v>
-      </c>
-      <c r="G75" s="1" t="s">
-        <v>273</v>
-      </c>
-      <c r="H75" s="1" t="s">
-        <v>274</v>
-      </c>
-      <c r="I75" s="1" t="s">
-        <v>275</v>
-      </c>
-      <c r="J75" s="1" t="s">
-        <v>276</v>
-      </c>
-      <c r="K75" s="1" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="76" ht="15.75" customHeight="1">
-      <c r="B76" s="1" t="s">
-        <v>278</v>
-      </c>
-      <c r="C76" s="1" t="s">
-        <v>279</v>
-      </c>
-      <c r="D76" s="1" t="s">
-        <v>280</v>
-      </c>
-      <c r="E76" s="1" t="s">
-        <v>281</v>
-      </c>
-      <c r="F76" s="1" t="s">
-        <v>282</v>
-      </c>
-      <c r="G76" s="1" t="s">
-        <v>283</v>
-      </c>
-      <c r="H76" s="1" t="s">
-        <v>284</v>
-      </c>
-      <c r="I76" s="1" t="s">
-        <v>285</v>
-      </c>
-      <c r="J76" s="1" t="s">
-        <v>286</v>
-      </c>
-      <c r="K76" s="1" t="s">
-        <v>287</v>
-      </c>
-    </row>
-    <row r="77" ht="15.75" customHeight="1">
-      <c r="B77" s="1" t="s">
-        <v>268</v>
-      </c>
-      <c r="C77" s="1" t="s">
-        <v>269</v>
-      </c>
-      <c r="D77" s="1" t="s">
-        <v>288</v>
-      </c>
-      <c r="E77" s="1" t="s">
-        <v>289</v>
-      </c>
-      <c r="F77" s="1" t="s">
-        <v>290</v>
-      </c>
-      <c r="G77" s="1" t="s">
-        <v>291</v>
-      </c>
-      <c r="H77" s="1" t="s">
-        <v>292</v>
-      </c>
-      <c r="I77" s="1" t="s">
-        <v>293</v>
-      </c>
-      <c r="J77" s="1" t="s">
-        <v>294</v>
-      </c>
-      <c r="K77" s="1" t="s">
-        <v>295</v>
-      </c>
-    </row>
-    <row r="78" ht="15.75" customHeight="1">
-      <c r="B78" s="1" t="s">
-        <v>278</v>
-      </c>
-      <c r="C78" s="1" t="s">
-        <v>279</v>
-      </c>
-      <c r="D78" s="1" t="s">
-        <v>296</v>
-      </c>
-      <c r="E78" s="1" t="s">
-        <v>297</v>
-      </c>
-      <c r="F78" s="1" t="s">
-        <v>298</v>
-      </c>
-      <c r="G78" s="1" t="s">
-        <v>299</v>
-      </c>
-      <c r="H78" s="1" t="s">
-        <v>300</v>
-      </c>
-      <c r="I78" s="1" t="s">
-        <v>301</v>
-      </c>
-      <c r="J78" s="1" t="s">
-        <v>302</v>
-      </c>
-      <c r="K78" s="1" t="s">
-        <v>303</v>
-      </c>
-    </row>
-    <row r="79" ht="15.75" customHeight="1">
-      <c r="C79" s="1" t="s">
-        <v>304</v>
-      </c>
-      <c r="D79" s="1" t="s">
-        <v>305</v>
-      </c>
-      <c r="E79" s="1" t="s">
-        <v>213</v>
-      </c>
-      <c r="F79" s="1" t="s">
-        <v>306</v>
-      </c>
-      <c r="G79" s="1" t="s">
-        <v>307</v>
-      </c>
-      <c r="H79" s="1" t="s">
-        <v>308</v>
-      </c>
-      <c r="I79" s="1" t="s">
-        <v>309</v>
-      </c>
       <c r="J79" s="1" t="s">
-        <v>310</v>
+        <v>237</v>
       </c>
       <c r="K79" s="1" t="s">
-        <v>311</v>
+        <v>238</v>
       </c>
     </row>
     <row r="80" ht="15.75" customHeight="1">
       <c r="B80" s="1" t="s">
-        <v>312</v>
+        <v>239</v>
       </c>
       <c r="C80" s="1" t="s">
-        <v>313</v>
-      </c>
-      <c r="D80" s="1" t="s">
-        <v>222</v>
+        <v>240</v>
       </c>
       <c r="E80" s="1" t="s">
-        <v>223</v>
+        <v>241</v>
       </c>
       <c r="F80" s="1" t="s">
-        <v>314</v>
+        <v>242</v>
       </c>
       <c r="G80" s="1" t="s">
-        <v>315</v>
+        <v>243</v>
       </c>
       <c r="H80" s="1" t="s">
-        <v>316</v>
+        <v>244</v>
       </c>
       <c r="I80" s="1" t="s">
-        <v>317</v>
+        <v>245</v>
       </c>
       <c r="J80" s="1" t="s">
-        <v>318</v>
+        <v>246</v>
       </c>
       <c r="K80" s="1" t="s">
-        <v>319</v>
+        <v>247</v>
       </c>
     </row>
     <row r="81" ht="15.75" customHeight="1">
+      <c r="B81" s="1" t="s">
+        <v>248</v>
+      </c>
       <c r="C81" s="1" t="s">
-        <v>304</v>
+        <v>249</v>
       </c>
       <c r="D81" s="1" t="s">
-        <v>320</v>
+        <v>250</v>
       </c>
       <c r="E81" s="1" t="s">
-        <v>321</v>
+        <v>251</v>
       </c>
       <c r="F81" s="1" t="s">
-        <v>322</v>
+        <v>252</v>
       </c>
       <c r="G81" s="1" t="s">
-        <v>323</v>
+        <v>253</v>
       </c>
       <c r="H81" s="1" t="s">
-        <v>324</v>
+        <v>254</v>
       </c>
       <c r="I81" s="1" t="s">
-        <v>325</v>
+        <v>255</v>
       </c>
       <c r="J81" s="1" t="s">
-        <v>326</v>
+        <v>256</v>
       </c>
       <c r="K81" s="1" t="s">
-        <v>327</v>
+        <v>257</v>
       </c>
     </row>
     <row r="82" ht="15.75" customHeight="1">
       <c r="B82" s="1" t="s">
-        <v>312</v>
+        <v>258</v>
       </c>
       <c r="C82" s="1" t="s">
-        <v>313</v>
+        <v>259</v>
       </c>
       <c r="D82" s="1" t="s">
-        <v>328</v>
+        <v>260</v>
       </c>
       <c r="E82" s="1" t="s">
-        <v>233</v>
+        <v>261</v>
+      </c>
+      <c r="F82" s="1" t="s">
+        <v>262</v>
+      </c>
+      <c r="G82" s="1" t="s">
+        <v>263</v>
       </c>
       <c r="H82" s="1" t="s">
-        <v>329</v>
+        <v>264</v>
       </c>
       <c r="I82" s="1" t="s">
-        <v>330</v>
+        <v>265</v>
       </c>
       <c r="J82" s="1" t="s">
-        <v>331</v>
+        <v>266</v>
       </c>
       <c r="K82" s="1" t="s">
-        <v>332</v>
+        <v>267</v>
       </c>
     </row>
     <row r="83" ht="15.75" customHeight="1">
-      <c r="B83" s="1" t="s">
-        <v>333</v>
-      </c>
       <c r="C83" s="1" t="s">
-        <v>334</v>
+        <v>268</v>
       </c>
       <c r="E83" s="1" t="s">
-        <v>249</v>
+        <v>269</v>
+      </c>
+      <c r="F83" s="1" t="s">
+        <v>270</v>
+      </c>
+      <c r="G83" s="1" t="s">
+        <v>271</v>
       </c>
       <c r="H83" s="1" t="s">
-        <v>335</v>
+        <v>272</v>
       </c>
       <c r="I83" s="1" t="s">
-        <v>336</v>
+        <v>273</v>
       </c>
       <c r="J83" s="1" t="s">
-        <v>337</v>
+        <v>274</v>
       </c>
       <c r="K83" s="1" t="s">
-        <v>338</v>
+        <v>275</v>
       </c>
     </row>
     <row r="84" ht="15.75" customHeight="1">
-      <c r="B84" s="1" t="s">
-        <v>339</v>
-      </c>
       <c r="C84" s="1" t="s">
-        <v>340</v>
+        <v>276</v>
       </c>
       <c r="E84" s="1" t="s">
-        <v>341</v>
+        <v>277</v>
+      </c>
+      <c r="F84" s="1" t="s">
+        <v>278</v>
+      </c>
+      <c r="G84" s="1" t="s">
+        <v>279</v>
       </c>
       <c r="H84" s="1" t="s">
-        <v>342</v>
+        <v>280</v>
       </c>
       <c r="I84" s="1" t="s">
-        <v>343</v>
+        <v>281</v>
       </c>
       <c r="J84" s="1" t="s">
-        <v>344</v>
+        <v>282</v>
       </c>
       <c r="K84" s="1" t="s">
-        <v>345</v>
+        <v>283</v>
       </c>
     </row>
     <row r="85" ht="15.75" customHeight="1">
-      <c r="B85" s="1" t="s">
-        <v>333</v>
-      </c>
       <c r="C85" s="1" t="s">
-        <v>334</v>
-      </c>
-      <c r="D85" s="1" t="s">
-        <v>280</v>
+        <v>268</v>
       </c>
       <c r="E85" s="1" t="s">
-        <v>281</v>
+        <v>284</v>
+      </c>
+      <c r="F85" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="G85" s="1" t="s">
+        <v>286</v>
       </c>
       <c r="H85" s="1" t="s">
-        <v>346</v>
+        <v>287</v>
       </c>
       <c r="I85" s="1" t="s">
-        <v>347</v>
+        <v>288</v>
       </c>
       <c r="J85" s="1" t="s">
-        <v>348</v>
+        <v>289</v>
       </c>
       <c r="K85" s="1" t="s">
-        <v>349</v>
+        <v>290</v>
       </c>
     </row>
     <row r="86" ht="15.75" customHeight="1">
-      <c r="B86" s="1" t="s">
-        <v>339</v>
-      </c>
       <c r="C86" s="1" t="s">
-        <v>340</v>
-      </c>
-      <c r="D86" s="1" t="s">
+        <v>276</v>
+      </c>
+      <c r="E86" s="1" t="s">
+        <v>291</v>
+      </c>
+      <c r="F86" s="1" t="s">
+        <v>292</v>
+      </c>
+      <c r="G86" s="1" t="s">
+        <v>293</v>
+      </c>
+      <c r="H86" s="1" t="s">
+        <v>287</v>
+      </c>
+      <c r="I86" s="1" t="s">
         <v>288</v>
       </c>
-      <c r="E86" s="1" t="s">
-        <v>289</v>
-      </c>
-      <c r="H86" s="1" t="s">
-        <v>350</v>
-      </c>
-      <c r="I86" s="1" t="s">
-        <v>351</v>
-      </c>
       <c r="J86" s="1" t="s">
-        <v>352</v>
+        <v>294</v>
       </c>
       <c r="K86" s="1" t="s">
-        <v>353</v>
+        <v>295</v>
       </c>
     </row>
     <row r="87" ht="15.75" customHeight="1">
       <c r="B87" s="1" t="s">
-        <v>354</v>
+        <v>296</v>
       </c>
       <c r="C87" s="1" t="s">
-        <v>355</v>
+        <v>297</v>
       </c>
       <c r="D87" s="1" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="E87" s="1" t="s">
-        <v>297</v>
+        <v>299</v>
+      </c>
+      <c r="F87" s="1" t="s">
+        <v>300</v>
+      </c>
+      <c r="G87" s="1" t="s">
+        <v>301</v>
       </c>
       <c r="H87" s="1" t="s">
-        <v>356</v>
+        <v>302</v>
       </c>
       <c r="I87" s="1" t="s">
-        <v>357</v>
+        <v>303</v>
       </c>
       <c r="J87" s="1" t="s">
-        <v>358</v>
+        <v>304</v>
       </c>
       <c r="K87" s="1" t="s">
-        <v>359</v>
+        <v>305</v>
       </c>
     </row>
     <row r="88" ht="15.75" customHeight="1">
+      <c r="B88" s="1" t="s">
+        <v>306</v>
+      </c>
       <c r="C88" s="1" t="s">
-        <v>360</v>
+        <v>307</v>
+      </c>
+      <c r="D88" s="1" t="s">
+        <v>308</v>
       </c>
       <c r="E88" s="1" t="s">
-        <v>213</v>
+        <v>309</v>
+      </c>
+      <c r="F88" s="1" t="s">
+        <v>310</v>
+      </c>
+      <c r="G88" s="1" t="s">
+        <v>311</v>
       </c>
       <c r="H88" s="1" t="s">
-        <v>361</v>
+        <v>312</v>
       </c>
       <c r="I88" s="1" t="s">
-        <v>362</v>
+        <v>313</v>
       </c>
       <c r="J88" s="1" t="s">
-        <v>363</v>
+        <v>314</v>
       </c>
       <c r="K88" s="1" t="s">
-        <v>364</v>
+        <v>315</v>
       </c>
     </row>
     <row r="89" ht="15.75" customHeight="1">
       <c r="B89" s="1" t="s">
-        <v>354</v>
+        <v>296</v>
       </c>
       <c r="C89" s="1" t="s">
-        <v>355</v>
+        <v>297</v>
       </c>
       <c r="D89" s="1" t="s">
-        <v>222</v>
+        <v>316</v>
       </c>
       <c r="E89" s="1" t="s">
-        <v>223</v>
+        <v>317</v>
+      </c>
+      <c r="F89" s="1" t="s">
+        <v>318</v>
+      </c>
+      <c r="G89" s="1" t="s">
+        <v>319</v>
       </c>
       <c r="H89" s="1" t="s">
-        <v>365</v>
+        <v>320</v>
       </c>
       <c r="I89" s="1" t="s">
-        <v>366</v>
+        <v>321</v>
       </c>
       <c r="J89" s="1" t="s">
-        <v>367</v>
+        <v>322</v>
       </c>
       <c r="K89" s="1" t="s">
-        <v>368</v>
+        <v>323</v>
       </c>
     </row>
     <row r="90" ht="15.75" customHeight="1">
       <c r="B90" s="1" t="s">
-        <v>369</v>
+        <v>306</v>
       </c>
       <c r="C90" s="1" t="s">
-        <v>370</v>
+        <v>307</v>
       </c>
       <c r="D90" s="1" t="s">
-        <v>320</v>
+        <v>324</v>
       </c>
       <c r="E90" s="1" t="s">
-        <v>321</v>
+        <v>325</v>
+      </c>
+      <c r="F90" s="1" t="s">
+        <v>326</v>
+      </c>
+      <c r="G90" s="1" t="s">
+        <v>327</v>
       </c>
       <c r="H90" s="1" t="s">
-        <v>371</v>
+        <v>328</v>
       </c>
       <c r="I90" s="1" t="s">
-        <v>372</v>
+        <v>329</v>
       </c>
       <c r="J90" s="1" t="s">
-        <v>373</v>
+        <v>330</v>
       </c>
       <c r="K90" s="1" t="s">
-        <v>374</v>
+        <v>331</v>
       </c>
     </row>
     <row r="91" ht="15.75" customHeight="1">
-      <c r="B91" s="1" t="s">
-        <v>375</v>
-      </c>
       <c r="C91" s="1" t="s">
-        <v>376</v>
+        <v>332</v>
       </c>
       <c r="D91" s="1" t="s">
-        <v>232</v>
+        <v>333</v>
       </c>
       <c r="E91" s="1" t="s">
-        <v>233</v>
+        <v>241</v>
+      </c>
+      <c r="F91" s="1" t="s">
+        <v>334</v>
+      </c>
+      <c r="G91" s="1" t="s">
+        <v>335</v>
       </c>
       <c r="H91" s="1" t="s">
-        <v>377</v>
+        <v>336</v>
       </c>
       <c r="I91" s="1" t="s">
-        <v>378</v>
+        <v>337</v>
+      </c>
+      <c r="J91" s="1" t="s">
+        <v>338</v>
+      </c>
+      <c r="K91" s="1" t="s">
+        <v>339</v>
       </c>
     </row>
     <row r="92" ht="15.75" customHeight="1">
       <c r="B92" s="1" t="s">
-        <v>379</v>
+        <v>340</v>
       </c>
       <c r="C92" s="1" t="s">
-        <v>379</v>
+        <v>341</v>
       </c>
       <c r="D92" s="1" t="s">
-        <v>380</v>
+        <v>250</v>
       </c>
       <c r="E92" s="1" t="s">
-        <v>241</v>
+        <v>251</v>
+      </c>
+      <c r="F92" s="1" t="s">
+        <v>342</v>
+      </c>
+      <c r="G92" s="1" t="s">
+        <v>343</v>
       </c>
       <c r="H92" s="1" t="s">
-        <v>381</v>
+        <v>344</v>
       </c>
       <c r="I92" s="1" t="s">
-        <v>382</v>
+        <v>345</v>
+      </c>
+      <c r="J92" s="1" t="s">
+        <v>346</v>
+      </c>
+      <c r="K92" s="1" t="s">
+        <v>347</v>
       </c>
     </row>
     <row r="93" ht="15.75" customHeight="1">
-      <c r="B93" s="1" t="s">
-        <v>375</v>
-      </c>
       <c r="C93" s="1" t="s">
-        <v>376</v>
+        <v>332</v>
       </c>
       <c r="D93" s="1" t="s">
-        <v>383</v>
+        <v>348</v>
       </c>
       <c r="E93" s="1" t="s">
-        <v>384</v>
+        <v>349</v>
+      </c>
+      <c r="F93" s="1" t="s">
+        <v>350</v>
+      </c>
+      <c r="G93" s="1" t="s">
+        <v>351</v>
       </c>
       <c r="H93" s="1" t="s">
-        <v>385</v>
+        <v>352</v>
       </c>
       <c r="I93" s="1" t="s">
-        <v>386</v>
+        <v>353</v>
+      </c>
+      <c r="J93" s="1" t="s">
+        <v>354</v>
+      </c>
+      <c r="K93" s="1" t="s">
+        <v>355</v>
       </c>
     </row>
     <row r="94" ht="15.75" customHeight="1">
       <c r="B94" s="1" t="s">
-        <v>379</v>
+        <v>340</v>
       </c>
       <c r="C94" s="1" t="s">
-        <v>379</v>
+        <v>341</v>
       </c>
       <c r="D94" s="1" t="s">
-        <v>387</v>
+        <v>356</v>
       </c>
       <c r="E94" s="1" t="s">
-        <v>388</v>
+        <v>261</v>
+      </c>
+      <c r="H94" s="1" t="s">
+        <v>357</v>
+      </c>
+      <c r="I94" s="1" t="s">
+        <v>358</v>
+      </c>
+      <c r="J94" s="1" t="s">
+        <v>359</v>
+      </c>
+      <c r="K94" s="1" t="s">
+        <v>360</v>
       </c>
     </row>
     <row r="95" ht="15.75" customHeight="1">
       <c r="B95" s="1" t="s">
-        <v>389</v>
+        <v>361</v>
       </c>
       <c r="C95" s="1" t="s">
-        <v>248</v>
+        <v>362</v>
       </c>
       <c r="E95" s="1" t="s">
-        <v>390</v>
+        <v>277</v>
+      </c>
+      <c r="H95" s="1" t="s">
+        <v>363</v>
+      </c>
+      <c r="I95" s="1" t="s">
+        <v>364</v>
+      </c>
+      <c r="J95" s="1" t="s">
+        <v>365</v>
+      </c>
+      <c r="K95" s="1" t="s">
+        <v>366</v>
       </c>
     </row>
     <row r="96" ht="15.75" customHeight="1">
       <c r="B96" s="1" t="s">
-        <v>391</v>
+        <v>367</v>
       </c>
       <c r="C96" s="1" t="s">
-        <v>392</v>
-      </c>
-      <c r="D96" s="1" t="s">
-        <v>393</v>
+        <v>368</v>
       </c>
       <c r="E96" s="1" t="s">
-        <v>394</v>
+        <v>369</v>
+      </c>
+      <c r="H96" s="1" t="s">
+        <v>370</v>
+      </c>
+      <c r="I96" s="1" t="s">
+        <v>371</v>
+      </c>
+      <c r="J96" s="1" t="s">
+        <v>372</v>
+      </c>
+      <c r="K96" s="1" t="s">
+        <v>373</v>
       </c>
     </row>
     <row r="97" ht="15.75" customHeight="1">
       <c r="B97" s="1" t="s">
-        <v>395</v>
+        <v>361</v>
       </c>
       <c r="C97" s="1" t="s">
-        <v>396</v>
+        <v>362</v>
       </c>
       <c r="D97" s="1" t="s">
-        <v>278</v>
+        <v>308</v>
       </c>
       <c r="E97" s="1" t="s">
-        <v>279</v>
+        <v>309</v>
+      </c>
+      <c r="H97" s="1" t="s">
+        <v>374</v>
+      </c>
+      <c r="I97" s="1" t="s">
+        <v>375</v>
+      </c>
+      <c r="J97" s="1" t="s">
+        <v>376</v>
+      </c>
+      <c r="K97" s="1" t="s">
+        <v>377</v>
       </c>
     </row>
     <row r="98" ht="15.75" customHeight="1">
       <c r="B98" s="1" t="s">
-        <v>397</v>
+        <v>367</v>
       </c>
       <c r="C98" s="1" t="s">
-        <v>398</v>
+        <v>368</v>
       </c>
       <c r="D98" s="1" t="s">
-        <v>270</v>
+        <v>316</v>
       </c>
       <c r="E98" s="1" t="s">
-        <v>271</v>
+        <v>317</v>
+      </c>
+      <c r="H98" s="1" t="s">
+        <v>378</v>
+      </c>
+      <c r="I98" s="1" t="s">
+        <v>379</v>
+      </c>
+      <c r="J98" s="1" t="s">
+        <v>380</v>
+      </c>
+      <c r="K98" s="1" t="s">
+        <v>381</v>
       </c>
     </row>
     <row r="99" ht="15.75" customHeight="1">
       <c r="B99" s="1" t="s">
+        <v>382</v>
+      </c>
+      <c r="C99" s="1" t="s">
+        <v>383</v>
+      </c>
+      <c r="D99" s="1" t="s">
+        <v>324</v>
+      </c>
+      <c r="E99" s="1" t="s">
+        <v>325</v>
+      </c>
+      <c r="H99" s="1" t="s">
+        <v>384</v>
+      </c>
+      <c r="I99" s="1" t="s">
+        <v>385</v>
+      </c>
+      <c r="J99" s="1" t="s">
+        <v>386</v>
+      </c>
+      <c r="K99" s="1" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="100" ht="15.75" customHeight="1">
+      <c r="C100" s="1" t="s">
+        <v>388</v>
+      </c>
+      <c r="E100" s="1" t="s">
+        <v>241</v>
+      </c>
+      <c r="H100" s="1" t="s">
+        <v>389</v>
+      </c>
+      <c r="I100" s="1" t="s">
+        <v>390</v>
+      </c>
+      <c r="J100" s="1" t="s">
+        <v>391</v>
+      </c>
+      <c r="K100" s="1" t="s">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="101" ht="15.75" customHeight="1">
+      <c r="B101" s="1" t="s">
+        <v>382</v>
+      </c>
+      <c r="C101" s="1" t="s">
+        <v>383</v>
+      </c>
+      <c r="D101" s="1" t="s">
+        <v>250</v>
+      </c>
+      <c r="E101" s="1" t="s">
+        <v>251</v>
+      </c>
+      <c r="H101" s="1" t="s">
+        <v>393</v>
+      </c>
+      <c r="I101" s="1" t="s">
+        <v>394</v>
+      </c>
+      <c r="J101" s="1" t="s">
+        <v>395</v>
+      </c>
+      <c r="K101" s="1" t="s">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="102" ht="15.75" customHeight="1">
+      <c r="B102" s="1" t="s">
+        <v>397</v>
+      </c>
+      <c r="C102" s="1" t="s">
+        <v>398</v>
+      </c>
+      <c r="D102" s="1" t="s">
+        <v>348</v>
+      </c>
+      <c r="E102" s="1" t="s">
+        <v>349</v>
+      </c>
+      <c r="H102" s="1" t="s">
         <v>399</v>
       </c>
-      <c r="C99" s="1" t="s">
+      <c r="I102" s="1" t="s">
         <v>400</v>
       </c>
-      <c r="D99" s="1" t="s">
+      <c r="J102" s="1" t="s">
         <v>401</v>
       </c>
-      <c r="E99" s="1" t="s">
+      <c r="K102" s="1" t="s">
         <v>402</v>
       </c>
     </row>
-    <row r="100" ht="15.75" customHeight="1">
-      <c r="D100" s="1" t="s">
-        <v>339</v>
-      </c>
-      <c r="E100" s="1" t="s">
-        <v>340</v>
-      </c>
-    </row>
-    <row r="101" ht="15.75" customHeight="1">
-      <c r="D101" s="1" t="s">
+    <row r="103" ht="15.75" customHeight="1">
+      <c r="B103" s="1" t="s">
         <v>403</v>
       </c>
-      <c r="E101" s="1" t="s">
+      <c r="C103" s="1" t="s">
         <v>404</v>
       </c>
-    </row>
-    <row r="102" ht="15.75" customHeight="1">
-      <c r="D102" s="1" t="s">
+      <c r="D103" s="1" t="s">
+        <v>260</v>
+      </c>
+      <c r="E103" s="1" t="s">
+        <v>261</v>
+      </c>
+      <c r="H103" s="1" t="s">
         <v>405</v>
       </c>
-      <c r="E102" s="1" t="s">
-        <v>390</v>
-      </c>
-    </row>
-    <row r="103" ht="15.75" customHeight="1">
-      <c r="D103" s="1" t="s">
-        <v>393</v>
-      </c>
-      <c r="E103" s="1" t="s">
-        <v>394</v>
+      <c r="I103" s="1" t="s">
+        <v>406</v>
       </c>
     </row>
     <row r="104" ht="15.75" customHeight="1">
+      <c r="B104" s="1" t="s">
+        <v>407</v>
+      </c>
+      <c r="C104" s="1" t="s">
+        <v>407</v>
+      </c>
       <c r="D104" s="1" t="s">
-        <v>278</v>
+        <v>408</v>
       </c>
       <c r="E104" s="1" t="s">
-        <v>279</v>
+        <v>269</v>
+      </c>
+      <c r="H104" s="1" t="s">
+        <v>409</v>
+      </c>
+      <c r="I104" s="1" t="s">
+        <v>410</v>
       </c>
     </row>
     <row r="105" ht="15.75" customHeight="1">
+      <c r="B105" s="1" t="s">
+        <v>403</v>
+      </c>
+      <c r="C105" s="1" t="s">
+        <v>404</v>
+      </c>
       <c r="D105" s="1" t="s">
-        <v>270</v>
+        <v>411</v>
       </c>
       <c r="E105" s="1" t="s">
-        <v>271</v>
+        <v>412</v>
+      </c>
+      <c r="H105" s="1" t="s">
+        <v>413</v>
+      </c>
+      <c r="I105" s="1" t="s">
+        <v>414</v>
       </c>
     </row>
     <row r="106" ht="15.75" customHeight="1">
+      <c r="B106" s="1" t="s">
+        <v>407</v>
+      </c>
+      <c r="C106" s="1" t="s">
+        <v>407</v>
+      </c>
       <c r="D106" s="1" t="s">
-        <v>401</v>
+        <v>415</v>
       </c>
       <c r="E106" s="1" t="s">
-        <v>402</v>
+        <v>416</v>
       </c>
     </row>
     <row r="107" ht="15.75" customHeight="1">
-      <c r="D107" s="1" t="s">
-        <v>339</v>
+      <c r="B107" s="1" t="s">
+        <v>417</v>
+      </c>
+      <c r="C107" s="1" t="s">
+        <v>276</v>
       </c>
       <c r="E107" s="1" t="s">
-        <v>340</v>
-      </c>
-    </row>
-    <row r="108" ht="15.75" customHeight="1"/>
-    <row r="109" ht="15.75" customHeight="1"/>
-    <row r="110" ht="15.75" customHeight="1"/>
-    <row r="111" ht="15.75" customHeight="1"/>
-    <row r="112" ht="15.75" customHeight="1"/>
-    <row r="113" ht="15.75" customHeight="1"/>
-    <row r="114" ht="15.75" customHeight="1"/>
-    <row r="115" ht="15.75" customHeight="1"/>
-    <row r="116" ht="15.75" customHeight="1"/>
-    <row r="117" ht="15.75" customHeight="1"/>
-    <row r="118" ht="15.75" customHeight="1"/>
-    <row r="119" ht="15.75" customHeight="1"/>
+        <v>418</v>
+      </c>
+    </row>
+    <row r="108" ht="15.75" customHeight="1">
+      <c r="B108" s="1" t="s">
+        <v>419</v>
+      </c>
+      <c r="C108" s="1" t="s">
+        <v>420</v>
+      </c>
+      <c r="D108" s="1" t="s">
+        <v>421</v>
+      </c>
+      <c r="E108" s="1" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="109" ht="15.75" customHeight="1">
+      <c r="B109" s="1" t="s">
+        <v>423</v>
+      </c>
+      <c r="C109" s="1" t="s">
+        <v>424</v>
+      </c>
+      <c r="D109" s="1" t="s">
+        <v>306</v>
+      </c>
+      <c r="E109" s="1" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="110" ht="15.75" customHeight="1">
+      <c r="B110" s="1" t="s">
+        <v>425</v>
+      </c>
+      <c r="C110" s="1" t="s">
+        <v>426</v>
+      </c>
+      <c r="D110" s="1" t="s">
+        <v>298</v>
+      </c>
+      <c r="E110" s="1" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="111" ht="15.75" customHeight="1">
+      <c r="B111" s="1" t="s">
+        <v>427</v>
+      </c>
+      <c r="C111" s="1" t="s">
+        <v>428</v>
+      </c>
+      <c r="D111" s="1" t="s">
+        <v>429</v>
+      </c>
+      <c r="E111" s="1" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="112" ht="15.75" customHeight="1">
+      <c r="D112" s="1" t="s">
+        <v>367</v>
+      </c>
+      <c r="E112" s="1" t="s">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="113" ht="15.75" customHeight="1">
+      <c r="D113" s="1" t="s">
+        <v>431</v>
+      </c>
+      <c r="E113" s="1" t="s">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="114" ht="15.75" customHeight="1">
+      <c r="D114" s="1" t="s">
+        <v>433</v>
+      </c>
+      <c r="E114" s="1" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="115" ht="15.75" customHeight="1">
+      <c r="D115" s="1" t="s">
+        <v>421</v>
+      </c>
+      <c r="E115" s="1" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="116" ht="15.75" customHeight="1">
+      <c r="D116" s="1" t="s">
+        <v>306</v>
+      </c>
+      <c r="E116" s="1" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="117" ht="15.75" customHeight="1">
+      <c r="D117" s="1" t="s">
+        <v>298</v>
+      </c>
+      <c r="E117" s="1" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="118" ht="15.75" customHeight="1">
+      <c r="D118" s="1" t="s">
+        <v>429</v>
+      </c>
+      <c r="E118" s="1" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="119" ht="15.75" customHeight="1">
+      <c r="D119" s="1" t="s">
+        <v>367</v>
+      </c>
+      <c r="E119" s="1" t="s">
+        <v>368</v>
+      </c>
+    </row>
     <row r="120" ht="15.75" customHeight="1"/>
     <row r="121" ht="15.75" customHeight="1"/>
     <row r="122" ht="15.75" customHeight="1"/>
@@ -4146,8 +4385,20 @@
     <row r="978" ht="15.75" customHeight="1"/>
     <row r="979" ht="15.75" customHeight="1"/>
     <row r="980" ht="15.75" customHeight="1"/>
+    <row r="981" ht="15.75" customHeight="1"/>
+    <row r="982" ht="15.75" customHeight="1"/>
+    <row r="983" ht="15.75" customHeight="1"/>
+    <row r="984" ht="15.75" customHeight="1"/>
+    <row r="985" ht="15.75" customHeight="1"/>
+    <row r="986" ht="15.75" customHeight="1"/>
+    <row r="987" ht="15.75" customHeight="1"/>
+    <row r="988" ht="15.75" customHeight="1"/>
+    <row r="989" ht="15.75" customHeight="1"/>
+    <row r="990" ht="15.75" customHeight="1"/>
+    <row r="991" ht="15.75" customHeight="1"/>
+    <row r="992" ht="15.75" customHeight="1"/>
   </sheetData>
-  <mergeCells count="60">
+  <mergeCells count="73">
     <mergeCell ref="H20:I20"/>
     <mergeCell ref="H31:I31"/>
     <mergeCell ref="H34:I34"/>
@@ -4160,17 +4411,28 @@
     <mergeCell ref="H19:I19"/>
     <mergeCell ref="G29:G41"/>
     <mergeCell ref="H36:I36"/>
-    <mergeCell ref="B61:C61"/>
-    <mergeCell ref="B62:C62"/>
-    <mergeCell ref="D62:E62"/>
-    <mergeCell ref="D64:E64"/>
-    <mergeCell ref="H49:I49"/>
-    <mergeCell ref="G57:K66"/>
-    <mergeCell ref="B59:C59"/>
-    <mergeCell ref="D59:E59"/>
-    <mergeCell ref="B60:C60"/>
-    <mergeCell ref="D60:E60"/>
-    <mergeCell ref="D61:E61"/>
+    <mergeCell ref="E44:F44"/>
+    <mergeCell ref="E47:F47"/>
+    <mergeCell ref="E48:F48"/>
+    <mergeCell ref="H32:I32"/>
+    <mergeCell ref="H33:I33"/>
+    <mergeCell ref="G42:G49"/>
+    <mergeCell ref="H43:I43"/>
+    <mergeCell ref="H44:I44"/>
+    <mergeCell ref="H45:I45"/>
+    <mergeCell ref="H46:I46"/>
+    <mergeCell ref="H48:I48"/>
+    <mergeCell ref="B73:C73"/>
+    <mergeCell ref="B74:C74"/>
+    <mergeCell ref="D74:E74"/>
+    <mergeCell ref="D76:E76"/>
+    <mergeCell ref="H61:I61"/>
+    <mergeCell ref="G69:K78"/>
+    <mergeCell ref="B71:C71"/>
+    <mergeCell ref="D71:E71"/>
+    <mergeCell ref="B72:C72"/>
+    <mergeCell ref="D72:E72"/>
+    <mergeCell ref="D73:E73"/>
     <mergeCell ref="E7:F7"/>
     <mergeCell ref="H7:I7"/>
     <mergeCell ref="E8:F8"/>
@@ -4189,25 +4451,27 @@
     <mergeCell ref="E5:F5"/>
     <mergeCell ref="E6:F6"/>
     <mergeCell ref="H9:I9"/>
-    <mergeCell ref="D44:E44"/>
-    <mergeCell ref="D45:E45"/>
-    <mergeCell ref="D46:E46"/>
+    <mergeCell ref="E45:F45"/>
+    <mergeCell ref="E46:F46"/>
+    <mergeCell ref="G50:G53"/>
+    <mergeCell ref="D56:E56"/>
+    <mergeCell ref="D57:E57"/>
+    <mergeCell ref="D58:E58"/>
     <mergeCell ref="H21:I21"/>
     <mergeCell ref="H22:I22"/>
-    <mergeCell ref="G42:G56"/>
-    <mergeCell ref="H45:I45"/>
-    <mergeCell ref="H46:I46"/>
-    <mergeCell ref="H47:I47"/>
-    <mergeCell ref="H48:I48"/>
-    <mergeCell ref="A67:A79"/>
-    <mergeCell ref="A80:A88"/>
+    <mergeCell ref="G54:G68"/>
+    <mergeCell ref="H57:I57"/>
+    <mergeCell ref="H58:I58"/>
+    <mergeCell ref="H59:I59"/>
+    <mergeCell ref="H60:I60"/>
+    <mergeCell ref="A79:A91"/>
+    <mergeCell ref="A92:A100"/>
     <mergeCell ref="A3:A15"/>
     <mergeCell ref="A16:A28"/>
     <mergeCell ref="A29:A41"/>
-    <mergeCell ref="A42:A54"/>
-    <mergeCell ref="A55:A66"/>
-    <mergeCell ref="H32:I32"/>
-    <mergeCell ref="H33:I33"/>
+    <mergeCell ref="A54:A66"/>
+    <mergeCell ref="A67:A78"/>
+    <mergeCell ref="A42:A53"/>
   </mergeCells>
   <printOptions/>
   <pageMargins bottom="1.0" footer="0.0" header="0.0" left="0.75" right="0.75" top="1.0"/>

</xml_diff>